<commit_message>
Actualizacion automatica -12-2025 17:38
</commit_message>
<xml_diff>
--- a/data/DSUBICI/RIVADAVIA.xlsx
+++ b/data/DSUBICI/RIVADAVIA.xlsx
@@ -483,7 +483,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2591</t>
+          <t>2591.0</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
@@ -522,7 +522,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>1344</t>
+          <t>1344.0</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
@@ -561,7 +561,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>1117</t>
+          <t>1117.0</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
@@ -604,7 +604,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>1102</t>
+          <t>1102.0</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
@@ -643,7 +643,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1087</t>
+          <t>1087.0</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
@@ -682,7 +682,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>1022</t>
+          <t>1022.0</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
@@ -721,7 +721,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>891</t>
+          <t>891.0</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
@@ -760,7 +760,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>850</t>
+          <t>850.0</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
@@ -799,7 +799,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>815</t>
+          <t>815.0</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
@@ -838,7 +838,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>721</t>
+          <t>721.0</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
@@ -881,7 +881,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>629</t>
+          <t>629.0</t>
         </is>
       </c>
       <c r="C12" t="inlineStr"/>
@@ -924,7 +924,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>581</t>
+          <t>581.0</t>
         </is>
       </c>
       <c r="C13" t="inlineStr"/>
@@ -963,7 +963,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>512</t>
+          <t>512.0</t>
         </is>
       </c>
       <c r="C14" t="inlineStr"/>
@@ -1002,7 +1002,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>505</t>
+          <t>505.0</t>
         </is>
       </c>
       <c r="C15" t="inlineStr"/>
@@ -1041,7 +1041,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>498</t>
+          <t>498.0</t>
         </is>
       </c>
       <c r="C16" t="inlineStr"/>
@@ -1080,7 +1080,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>485</t>
+          <t>485.0</t>
         </is>
       </c>
       <c r="C17" t="inlineStr"/>
@@ -1119,7 +1119,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>463</t>
+          <t>463.0</t>
         </is>
       </c>
       <c r="C18" t="inlineStr"/>
@@ -1158,7 +1158,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>461</t>
+          <t>461.0</t>
         </is>
       </c>
       <c r="C19" t="inlineStr"/>
@@ -1197,7 +1197,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>456</t>
+          <t>456.0</t>
         </is>
       </c>
       <c r="C20" t="inlineStr"/>
@@ -1240,7 +1240,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>448</t>
+          <t>448.0</t>
         </is>
       </c>
       <c r="C21" t="inlineStr"/>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>411</t>
+          <t>411.0</t>
         </is>
       </c>
       <c r="C22" t="inlineStr"/>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>401</t>
+          <t>401.0</t>
         </is>
       </c>
       <c r="C23" t="inlineStr"/>
@@ -1361,7 +1361,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>374</t>
+          <t>374.0</t>
         </is>
       </c>
       <c r="C24" t="inlineStr"/>
@@ -1400,7 +1400,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>3613.</t>
+          <t>3613.0</t>
         </is>
       </c>
       <c r="C25" t="inlineStr"/>
@@ -1478,7 +1478,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>341</t>
+          <t>341.0</t>
         </is>
       </c>
       <c r="C27" t="inlineStr"/>
@@ -1517,7 +1517,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>340</t>
+          <t>340.0</t>
         </is>
       </c>
       <c r="C28" t="inlineStr"/>
@@ -1556,7 +1556,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>330</t>
+          <t>330.0</t>
         </is>
       </c>
       <c r="C29" t="inlineStr"/>
@@ -1595,7 +1595,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>314</t>
+          <t>314.0</t>
         </is>
       </c>
       <c r="C30" t="inlineStr"/>
@@ -1634,7 +1634,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>306</t>
+          <t>306.0</t>
         </is>
       </c>
       <c r="C31" t="inlineStr"/>
@@ -1790,7 +1790,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>283</t>
+          <t>283.0</t>
         </is>
       </c>
       <c r="C35" t="inlineStr"/>
@@ -1907,7 +1907,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>273</t>
+          <t>273.0</t>
         </is>
       </c>
       <c r="C38" t="inlineStr"/>
@@ -1946,7 +1946,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>270</t>
+          <t>270.0</t>
         </is>
       </c>
       <c r="C39" t="inlineStr"/>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>264</t>
+          <t>264.0</t>
         </is>
       </c>
       <c r="C40" t="inlineStr"/>
@@ -2024,7 +2024,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>259</t>
+          <t>259.0</t>
         </is>
       </c>
       <c r="C41" t="inlineStr"/>
@@ -2219,7 +2219,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>247.0</t>
         </is>
       </c>
       <c r="C46" t="inlineStr"/>
@@ -2297,7 +2297,7 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>247</t>
+          <t>247.0</t>
         </is>
       </c>
       <c r="C48" t="inlineStr"/>
@@ -2496,7 +2496,7 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>234</t>
+          <t>234.0</t>
         </is>
       </c>
       <c r="C53" t="inlineStr"/>
@@ -2656,7 +2656,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>203.0</t>
         </is>
       </c>
       <c r="C57" t="inlineStr"/>
@@ -2695,7 +2695,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>203</t>
+          <t>203.0</t>
         </is>
       </c>
       <c r="C58" t="inlineStr"/>
@@ -2812,7 +2812,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>201</t>
+          <t>201.0</t>
         </is>
       </c>
       <c r="C61" t="inlineStr"/>
@@ -2929,7 +2929,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>187</t>
+          <t>187.0</t>
         </is>
       </c>
       <c r="C64" t="inlineStr"/>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>173.0</t>
         </is>
       </c>
       <c r="C70" t="inlineStr"/>
@@ -3210,7 +3210,7 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>173</t>
+          <t>173.0</t>
         </is>
       </c>
       <c r="C71" t="inlineStr"/>
@@ -3448,7 +3448,7 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>162</t>
+          <t>162.0</t>
         </is>
       </c>
       <c r="C77" t="inlineStr"/>
@@ -3692,12 +3692,12 @@
       <c r="C83" t="inlineStr"/>
       <c r="D83" t="inlineStr">
         <is>
-          <t>ISABEL MARIA Y  LAURA VIÑAS</t>
+          <t>PROVINVEST</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>*</t>
+          <t>EXIMIA</t>
         </is>
       </c>
       <c r="F83" t="inlineStr"/>
@@ -3708,7 +3708,7 @@
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>#ffffff</t>
+          <t>#ffff00</t>
         </is>
       </c>
       <c r="I83" t="inlineStr">
@@ -4154,7 +4154,7 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>148.0</t>
         </is>
       </c>
       <c r="C95" t="inlineStr"/>
@@ -4634,7 +4634,7 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>128</t>
+          <t>128.0</t>
         </is>
       </c>
       <c r="C107" t="inlineStr"/>
@@ -4829,7 +4829,7 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>126</t>
+          <t>126.0</t>
         </is>
       </c>
       <c r="C112" t="inlineStr"/>
@@ -5102,7 +5102,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>118</t>
+          <t>118.0</t>
         </is>
       </c>
       <c r="C119" t="inlineStr"/>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>116</t>
+          <t>116.0</t>
         </is>
       </c>
       <c r="C121" t="inlineStr"/>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>109</t>
+          <t>109.0</t>
         </is>
       </c>
       <c r="C129" t="inlineStr"/>
@@ -5621,7 +5621,7 @@
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>106.0</t>
         </is>
       </c>
       <c r="C132" t="inlineStr"/>
@@ -5660,7 +5660,7 @@
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>106</t>
+          <t>106.0</t>
         </is>
       </c>
       <c r="C133" t="inlineStr"/>
@@ -5738,7 +5738,7 @@
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>104</t>
+          <t>104.0</t>
         </is>
       </c>
       <c r="C135" t="inlineStr"/>
@@ -7612,11 +7612,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I182" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I182" t="inlineStr"/>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -9726,11 +9722,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I236" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I236" t="inlineStr"/>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -12156,11 +12148,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I298" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I298" t="inlineStr"/>
     </row>
     <row r="299">
       <c r="A299" t="inlineStr">
@@ -12433,11 +12421,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I305" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I305" t="inlineStr"/>
     </row>
     <row r="306">
       <c r="A306" t="inlineStr">
@@ -21080,11 +21064,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I526" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I526" t="inlineStr"/>
     </row>
     <row r="527">
       <c r="A527" t="inlineStr">
@@ -21119,11 +21099,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I527" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I527" t="inlineStr"/>
     </row>
     <row r="528">
       <c r="A528" t="inlineStr">
@@ -22562,11 +22538,7 @@
           <t>#00ff00</t>
         </is>
       </c>
-      <c r="I564" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I564" t="inlineStr"/>
     </row>
     <row r="565">
       <c r="A565" t="inlineStr">
@@ -27772,11 +27744,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I698" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I698" t="inlineStr"/>
     </row>
     <row r="699">
       <c r="A699" t="inlineStr">
@@ -28162,11 +28130,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I708" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I708" t="inlineStr"/>
     </row>
     <row r="709">
       <c r="A709" t="inlineStr">
@@ -33357,11 +33321,7 @@
           <t>#ffffff</t>
         </is>
       </c>
-      <c r="I841" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I841" t="inlineStr"/>
     </row>
     <row r="842">
       <c r="A842" t="inlineStr">
@@ -43543,11 +43503,7 @@
           <t>#ff0000</t>
         </is>
       </c>
-      <c r="I1103" t="inlineStr">
-        <is>
-          <t>[]</t>
-        </is>
-      </c>
+      <c r="I1103" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>